<commit_message>
Rules pass (Template Rulebook 2026-10-29)
- Universal legend on every training sheet; prep = 1 warm-up set
- Sub-Level 3 PRACTICE TEST defined; progression-line choices are the member's pick
- "TEST DAY" -> "Boss Test" (tab + legend); one Boss Test closes Day 1 and Day 2
- Boss Test legend: 2 warm-up sets per test, exact standard once, already-passed tests count

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Z6iaoJGzk5zGc6QzZeS76
</commit_message>
<xml_diff>
--- a/Level2_Locomotion_Day1_SubLevel1_Micro_Cycles-2.xlsx
+++ b/Level2_Locomotion_Day1_SubLevel1_Micro_Cycles-2.xlsx
@@ -511,10 +511,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1" s="20">
+    <row r="2" ht="54" customHeight="1" s="20">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Self-paced — stay on each exercise until the standard is earned. Train inside the PRESCRIPTION range; the top of the range is the STANDARD. Hitting the standard = signal you may be ready to test. ○ = working grade, 0 = Foundation, 1·2 / 2·3 = carries in both sub-levels. PICK 1 = choose one. Every cell is a per-set prescription. Yellow TBD = no number in the source yet.</t>
+          <t>Self-paced. Train inside the PRESCRIPTION; its top is the STANDARD. One set at the standard = that exercise is passed. Clear a slot by passing 2 different exercises from its list (1 if it lists only one) — ○ 0 Foundations count, warm-ups/prep/activation/rotator don't. Clear every slot to move to the next phase. PICK 1 = choose one, PICK 2 = choose two. Every cell is a per-set prescription. Weighted rows: up to 1–2 warm-up sets below the range, then at least 1 set inside it. ○ = working grade, 0 = Foundation, 1·2 / 2·3 = carries in both sub-levels. Progression-line choices are your pick each session.</t>
         </is>
       </c>
     </row>

</xml_diff>